<commit_message>
Adding Ex4A Insert Records
</commit_message>
<xml_diff>
--- a/karaere_Ex3A_tables.xlsx
+++ b/karaere_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\onurkaraer\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981C00EB-CB62-435A-857C-F7660A492CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC6B9DC-E94C-4F94-B763-DCA7CF83683A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="2940" windowWidth="21600" windowHeight="11295" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t>customer_id</t>
   </si>
@@ -95,12 +95,50 @@
   </si>
   <si>
     <t>duration</t>
+  </si>
+  <si>
+    <t>Jillian Furey</t>
+  </si>
+  <si>
+    <t>1249 W Chase Ave</t>
+  </si>
+  <si>
+    <t>DOG-1</t>
+  </si>
+  <si>
+    <t>CUS-1</t>
+  </si>
+  <si>
+    <t>Darla</t>
+  </si>
+  <si>
+    <t>Poodle</t>
+  </si>
+  <si>
+    <t>WAL-1</t>
+  </si>
+  <si>
+    <t>Jason Parley</t>
+  </si>
+  <si>
+    <t>TR1234567890</t>
+  </si>
+  <si>
+    <t>Amex</t>
+  </si>
+  <si>
+    <t>W-00000001</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="168" formatCode="h:mm:ss;@"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -142,10 +180,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -426,17 +467,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.28515625" customWidth="1"/>
     <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -452,8 +493,22 @@
       <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="F1" t="s">
-        <v>1</v>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>3124457896</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -463,7 +518,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9B54C0C-379F-4F5A-92EB-DD6951B98EDC}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -490,6 +545,23 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2">
+        <v>4.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -497,7 +569,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB7700A1-D67C-4511-81D4-C88E1AFB3CC2}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -520,6 +592,20 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>3125568413</v>
+      </c>
+      <c r="D2">
+        <v>4.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -527,10 +613,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1284E666-7BD9-4B61-B87D-E301B67FD4AA}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -548,6 +635,20 @@
         <v>17</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>1234567890</v>
+      </c>
+      <c r="C2" s="3">
+        <v>98.15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -555,13 +656,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEB1A590-2084-4A0A-91D8-7023B05E2907}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -585,6 +686,26 @@
         <v>21</v>
       </c>
     </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46068</v>
+      </c>
+      <c r="E2" s="5">
+        <v>0.5625</v>
+      </c>
+      <c r="F2" s="5">
+        <v>4.5138888888888888E-2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>